<commit_message>
Fix incentive pot references and the per-KPI phasing check
- Earned-YTD used column H (Focus pot) instead of column G (Lead pot), so
  every quarterly payout was computed off the wrong pot; focus payout used
  column I (the Q1 factor) instead of H. Both now point at the right pots.
- A quarter beyond Setup!C5 earns nothing and reads "Chưa chốt" rather than
  "Behind"; Focus pays only once Q4 is closed. Headers say the totals are
  paid-to-date.
- The Weekly_Tracker check column pointed at the merged Emp Code cell, so it
  stayed blank for KPI 2-5 of each person; it now reads the block anchor.

Verified with audit.py (600 cross-sheet references) and check_values.py
(390 recomputed values, 16,989 formula cells evaluated, no formula errors).
LibreOffice recalc is unusable in this container - it hangs on a 4-cell file -
so the `formulas` engine was used instead.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LMAoye3x9B7d3mF4at83kf
</commit_message>
<xml_diff>
--- a/dulux-kpi-tracker/Dulux_Channel_KPI_Tracker_2026.xlsx
+++ b/dulux-kpi-tracker/Dulux_Channel_KPI_Tracker_2026.xlsx
@@ -2825,7 +2825,7 @@
         <v/>
       </c>
       <c r="I6" s="41">
-        <f>IF($A6="","",IF($G6=0,"chưa nhập FY target",IF(ROUND(H6-$G6,2)=0,"OK","Lệch "&amp;TEXT(H6-$G6,"#,##0"))))</f>
+        <f>IF($A$6="","",IF($G6=0,"chưa nhập FY target",IF(ROUND(H6-$G6,2)=0,"OK","Lệch "&amp;TEXT(H6-$G6,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J6" s="28" t="n">
@@ -3427,7 +3427,7 @@
         <v/>
       </c>
       <c r="I9" s="41">
-        <f>IF($A9="","",IF($G9=0,"chưa nhập FY target",IF(ROUND(H9-$G9,2)=0,"OK","Lệch "&amp;TEXT(H9-$G9,"#,##0"))))</f>
+        <f>IF($A$6="","",IF($G9=0,"chưa nhập FY target",IF(ROUND(H9-$G9,2)=0,"OK","Lệch "&amp;TEXT(H9-$G9,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J9" s="28" t="n">
@@ -4029,7 +4029,7 @@
         <v/>
       </c>
       <c r="I12" s="41">
-        <f>IF($A12="","",IF($G12=0,"chưa nhập FY target",IF(ROUND(H12-$G12,2)=0,"OK","Lệch "&amp;TEXT(H12-$G12,"#,##0"))))</f>
+        <f>IF($A$6="","",IF($G12=0,"chưa nhập FY target",IF(ROUND(H12-$G12,2)=0,"OK","Lệch "&amp;TEXT(H12-$G12,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J12" s="28" t="n">
@@ -4631,7 +4631,7 @@
         <v/>
       </c>
       <c r="I15" s="41">
-        <f>IF($A15="","",IF($G15=0,"chưa nhập FY target",IF(ROUND(H15-$G15,2)=0,"OK","Lệch "&amp;TEXT(H15-$G15,"#,##0"))))</f>
+        <f>IF($A$6="","",IF($G15=0,"chưa nhập FY target",IF(ROUND(H15-$G15,2)=0,"OK","Lệch "&amp;TEXT(H15-$G15,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J15" s="28" t="n">
@@ -5233,7 +5233,7 @@
         <v/>
       </c>
       <c r="I18" s="41">
-        <f>IF($A18="","",IF($G18=0,"chưa nhập FY target",IF(ROUND(H18-$G18,2)=0,"OK","Lệch "&amp;TEXT(H18-$G18,"#,##0"))))</f>
+        <f>IF($A$6="","",IF($G18=0,"chưa nhập FY target",IF(ROUND(H18-$G18,2)=0,"OK","Lệch "&amp;TEXT(H18-$G18,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J18" s="28" t="n">
@@ -5841,7 +5841,7 @@
         <v/>
       </c>
       <c r="I21" s="41">
-        <f>IF($A21="","",IF($G21=0,"chưa nhập FY target",IF(ROUND(H21-$G21,2)=0,"OK","Lệch "&amp;TEXT(H21-$G21,"#,##0"))))</f>
+        <f>IF($A$21="","",IF($G21=0,"chưa nhập FY target",IF(ROUND(H21-$G21,2)=0,"OK","Lệch "&amp;TEXT(H21-$G21,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J21" s="28" t="n">
@@ -6443,7 +6443,7 @@
         <v/>
       </c>
       <c r="I24" s="41">
-        <f>IF($A24="","",IF($G24=0,"chưa nhập FY target",IF(ROUND(H24-$G24,2)=0,"OK","Lệch "&amp;TEXT(H24-$G24,"#,##0"))))</f>
+        <f>IF($A$21="","",IF($G24=0,"chưa nhập FY target",IF(ROUND(H24-$G24,2)=0,"OK","Lệch "&amp;TEXT(H24-$G24,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J24" s="28" t="n">
@@ -7045,7 +7045,7 @@
         <v/>
       </c>
       <c r="I27" s="41">
-        <f>IF($A27="","",IF($G27=0,"chưa nhập FY target",IF(ROUND(H27-$G27,2)=0,"OK","Lệch "&amp;TEXT(H27-$G27,"#,##0"))))</f>
+        <f>IF($A$21="","",IF($G27=0,"chưa nhập FY target",IF(ROUND(H27-$G27,2)=0,"OK","Lệch "&amp;TEXT(H27-$G27,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J27" s="28" t="n">
@@ -7647,7 +7647,7 @@
         <v/>
       </c>
       <c r="I30" s="41">
-        <f>IF($A30="","",IF($G30=0,"chưa nhập FY target",IF(ROUND(H30-$G30,2)=0,"OK","Lệch "&amp;TEXT(H30-$G30,"#,##0"))))</f>
+        <f>IF($A$21="","",IF($G30=0,"chưa nhập FY target",IF(ROUND(H30-$G30,2)=0,"OK","Lệch "&amp;TEXT(H30-$G30,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J30" s="28" t="n">
@@ -8249,7 +8249,7 @@
         <v/>
       </c>
       <c r="I33" s="41">
-        <f>IF($A33="","",IF($G33=0,"chưa nhập FY target",IF(ROUND(H33-$G33,2)=0,"OK","Lệch "&amp;TEXT(H33-$G33,"#,##0"))))</f>
+        <f>IF($A$21="","",IF($G33=0,"chưa nhập FY target",IF(ROUND(H33-$G33,2)=0,"OK","Lệch "&amp;TEXT(H33-$G33,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J33" s="28" t="n">
@@ -8857,7 +8857,7 @@
         <v/>
       </c>
       <c r="I36" s="41">
-        <f>IF($A36="","",IF($G36=0,"chưa nhập FY target",IF(ROUND(H36-$G36,2)=0,"OK","Lệch "&amp;TEXT(H36-$G36,"#,##0"))))</f>
+        <f>IF($A$36="","",IF($G36=0,"chưa nhập FY target",IF(ROUND(H36-$G36,2)=0,"OK","Lệch "&amp;TEXT(H36-$G36,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J36" s="28" t="n">
@@ -9459,7 +9459,7 @@
         <v/>
       </c>
       <c r="I39" s="41">
-        <f>IF($A39="","",IF($G39=0,"chưa nhập FY target",IF(ROUND(H39-$G39,2)=0,"OK","Lệch "&amp;TEXT(H39-$G39,"#,##0"))))</f>
+        <f>IF($A$36="","",IF($G39=0,"chưa nhập FY target",IF(ROUND(H39-$G39,2)=0,"OK","Lệch "&amp;TEXT(H39-$G39,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J39" s="28" t="n">
@@ -10061,7 +10061,7 @@
         <v/>
       </c>
       <c r="I42" s="41">
-        <f>IF($A42="","",IF($G42=0,"chưa nhập FY target",IF(ROUND(H42-$G42,2)=0,"OK","Lệch "&amp;TEXT(H42-$G42,"#,##0"))))</f>
+        <f>IF($A$36="","",IF($G42=0,"chưa nhập FY target",IF(ROUND(H42-$G42,2)=0,"OK","Lệch "&amp;TEXT(H42-$G42,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J42" s="28" t="n">
@@ -10663,7 +10663,7 @@
         <v/>
       </c>
       <c r="I45" s="41">
-        <f>IF($A45="","",IF($G45=0,"chưa nhập FY target",IF(ROUND(H45-$G45,2)=0,"OK","Lệch "&amp;TEXT(H45-$G45,"#,##0"))))</f>
+        <f>IF($A$36="","",IF($G45=0,"chưa nhập FY target",IF(ROUND(H45-$G45,2)=0,"OK","Lệch "&amp;TEXT(H45-$G45,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J45" s="28" t="n">
@@ -11265,7 +11265,7 @@
         <v/>
       </c>
       <c r="I48" s="41">
-        <f>IF($A48="","",IF($G48=0,"chưa nhập FY target",IF(ROUND(H48-$G48,2)=0,"OK","Lệch "&amp;TEXT(H48-$G48,"#,##0"))))</f>
+        <f>IF($A$36="","",IF($G48=0,"chưa nhập FY target",IF(ROUND(H48-$G48,2)=0,"OK","Lệch "&amp;TEXT(H48-$G48,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J48" s="28" t="n">
@@ -11873,7 +11873,7 @@
         <v/>
       </c>
       <c r="I51" s="41">
-        <f>IF($A51="","",IF($G51=0,"chưa nhập FY target",IF(ROUND(H51-$G51,2)=0,"OK","Lệch "&amp;TEXT(H51-$G51,"#,##0"))))</f>
+        <f>IF($A$51="","",IF($G51=0,"chưa nhập FY target",IF(ROUND(H51-$G51,2)=0,"OK","Lệch "&amp;TEXT(H51-$G51,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J51" s="28" t="n">
@@ -12475,7 +12475,7 @@
         <v/>
       </c>
       <c r="I54" s="41">
-        <f>IF($A54="","",IF($G54=0,"chưa nhập FY target",IF(ROUND(H54-$G54,2)=0,"OK","Lệch "&amp;TEXT(H54-$G54,"#,##0"))))</f>
+        <f>IF($A$51="","",IF($G54=0,"chưa nhập FY target",IF(ROUND(H54-$G54,2)=0,"OK","Lệch "&amp;TEXT(H54-$G54,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J54" s="28" t="n">
@@ -13077,7 +13077,7 @@
         <v/>
       </c>
       <c r="I57" s="41">
-        <f>IF($A57="","",IF($G57=0,"chưa nhập FY target",IF(ROUND(H57-$G57,2)=0,"OK","Lệch "&amp;TEXT(H57-$G57,"#,##0"))))</f>
+        <f>IF($A$51="","",IF($G57=0,"chưa nhập FY target",IF(ROUND(H57-$G57,2)=0,"OK","Lệch "&amp;TEXT(H57-$G57,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J57" s="28" t="n">
@@ -13679,7 +13679,7 @@
         <v/>
       </c>
       <c r="I60" s="41">
-        <f>IF($A60="","",IF($G60=0,"chưa nhập FY target",IF(ROUND(H60-$G60,2)=0,"OK","Lệch "&amp;TEXT(H60-$G60,"#,##0"))))</f>
+        <f>IF($A$51="","",IF($G60=0,"chưa nhập FY target",IF(ROUND(H60-$G60,2)=0,"OK","Lệch "&amp;TEXT(H60-$G60,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J60" s="28" t="n">
@@ -14281,7 +14281,7 @@
         <v/>
       </c>
       <c r="I63" s="41">
-        <f>IF($A63="","",IF($G63=0,"chưa nhập FY target",IF(ROUND(H63-$G63,2)=0,"OK","Lệch "&amp;TEXT(H63-$G63,"#,##0"))))</f>
+        <f>IF($A$51="","",IF($G63=0,"chưa nhập FY target",IF(ROUND(H63-$G63,2)=0,"OK","Lệch "&amp;TEXT(H63-$G63,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J63" s="28" t="n">
@@ -14889,7 +14889,7 @@
         <v/>
       </c>
       <c r="I66" s="41">
-        <f>IF($A66="","",IF($G66=0,"chưa nhập FY target",IF(ROUND(H66-$G66,2)=0,"OK","Lệch "&amp;TEXT(H66-$G66,"#,##0"))))</f>
+        <f>IF($A$66="","",IF($G66=0,"chưa nhập FY target",IF(ROUND(H66-$G66,2)=0,"OK","Lệch "&amp;TEXT(H66-$G66,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J66" s="28" t="n">
@@ -15491,7 +15491,7 @@
         <v/>
       </c>
       <c r="I69" s="41">
-        <f>IF($A69="","",IF($G69=0,"chưa nhập FY target",IF(ROUND(H69-$G69,2)=0,"OK","Lệch "&amp;TEXT(H69-$G69,"#,##0"))))</f>
+        <f>IF($A$66="","",IF($G69=0,"chưa nhập FY target",IF(ROUND(H69-$G69,2)=0,"OK","Lệch "&amp;TEXT(H69-$G69,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J69" s="28" t="n">
@@ -16093,7 +16093,7 @@
         <v/>
       </c>
       <c r="I72" s="41">
-        <f>IF($A72="","",IF($G72=0,"chưa nhập FY target",IF(ROUND(H72-$G72,2)=0,"OK","Lệch "&amp;TEXT(H72-$G72,"#,##0"))))</f>
+        <f>IF($A$66="","",IF($G72=0,"chưa nhập FY target",IF(ROUND(H72-$G72,2)=0,"OK","Lệch "&amp;TEXT(H72-$G72,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J72" s="28" t="n">
@@ -16695,7 +16695,7 @@
         <v/>
       </c>
       <c r="I75" s="41">
-        <f>IF($A75="","",IF($G75=0,"chưa nhập FY target",IF(ROUND(H75-$G75,2)=0,"OK","Lệch "&amp;TEXT(H75-$G75,"#,##0"))))</f>
+        <f>IF($A$66="","",IF($G75=0,"chưa nhập FY target",IF(ROUND(H75-$G75,2)=0,"OK","Lệch "&amp;TEXT(H75-$G75,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J75" s="28" t="n">
@@ -17297,7 +17297,7 @@
         <v/>
       </c>
       <c r="I78" s="41">
-        <f>IF($A78="","",IF($G78=0,"chưa nhập FY target",IF(ROUND(H78-$G78,2)=0,"OK","Lệch "&amp;TEXT(H78-$G78,"#,##0"))))</f>
+        <f>IF($A$66="","",IF($G78=0,"chưa nhập FY target",IF(ROUND(H78-$G78,2)=0,"OK","Lệch "&amp;TEXT(H78-$G78,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J78" s="28" t="n">
@@ -17905,7 +17905,7 @@
         <v/>
       </c>
       <c r="I81" s="41">
-        <f>IF($A81="","",IF($G81=0,"chưa nhập FY target",IF(ROUND(H81-$G81,2)=0,"OK","Lệch "&amp;TEXT(H81-$G81,"#,##0"))))</f>
+        <f>IF($A$81="","",IF($G81=0,"chưa nhập FY target",IF(ROUND(H81-$G81,2)=0,"OK","Lệch "&amp;TEXT(H81-$G81,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J81" s="28" t="n">
@@ -18507,7 +18507,7 @@
         <v/>
       </c>
       <c r="I84" s="41">
-        <f>IF($A84="","",IF($G84=0,"chưa nhập FY target",IF(ROUND(H84-$G84,2)=0,"OK","Lệch "&amp;TEXT(H84-$G84,"#,##0"))))</f>
+        <f>IF($A$81="","",IF($G84=0,"chưa nhập FY target",IF(ROUND(H84-$G84,2)=0,"OK","Lệch "&amp;TEXT(H84-$G84,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J84" s="28" t="n">
@@ -19109,7 +19109,7 @@
         <v/>
       </c>
       <c r="I87" s="41">
-        <f>IF($A87="","",IF($G87=0,"chưa nhập FY target",IF(ROUND(H87-$G87,2)=0,"OK","Lệch "&amp;TEXT(H87-$G87,"#,##0"))))</f>
+        <f>IF($A$81="","",IF($G87=0,"chưa nhập FY target",IF(ROUND(H87-$G87,2)=0,"OK","Lệch "&amp;TEXT(H87-$G87,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J87" s="28" t="n">
@@ -19711,7 +19711,7 @@
         <v/>
       </c>
       <c r="I90" s="41">
-        <f>IF($A90="","",IF($G90=0,"chưa nhập FY target",IF(ROUND(H90-$G90,2)=0,"OK","Lệch "&amp;TEXT(H90-$G90,"#,##0"))))</f>
+        <f>IF($A$81="","",IF($G90=0,"chưa nhập FY target",IF(ROUND(H90-$G90,2)=0,"OK","Lệch "&amp;TEXT(H90-$G90,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J90" s="28" t="n">
@@ -20313,7 +20313,7 @@
         <v/>
       </c>
       <c r="I93" s="41">
-        <f>IF($A93="","",IF($G93=0,"chưa nhập FY target",IF(ROUND(H93-$G93,2)=0,"OK","Lệch "&amp;TEXT(H93-$G93,"#,##0"))))</f>
+        <f>IF($A$81="","",IF($G93=0,"chưa nhập FY target",IF(ROUND(H93-$G93,2)=0,"OK","Lệch "&amp;TEXT(H93-$G93,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J93" s="28" t="n">
@@ -20919,7 +20919,7 @@
         <v/>
       </c>
       <c r="I96" s="41">
-        <f>IF($A96="","",IF($G96=0,"chưa nhập FY target",IF(ROUND(H96-$G96,2)=0,"OK","Lệch "&amp;TEXT(H96-$G96,"#,##0"))))</f>
+        <f>IF($A$96="","",IF($G96=0,"chưa nhập FY target",IF(ROUND(H96-$G96,2)=0,"OK","Lệch "&amp;TEXT(H96-$G96,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J96" s="28" t="n"/>
@@ -21351,7 +21351,7 @@
         <v/>
       </c>
       <c r="I99" s="41">
-        <f>IF($A99="","",IF($G99=0,"chưa nhập FY target",IF(ROUND(H99-$G99,2)=0,"OK","Lệch "&amp;TEXT(H99-$G99,"#,##0"))))</f>
+        <f>IF($A$96="","",IF($G99=0,"chưa nhập FY target",IF(ROUND(H99-$G99,2)=0,"OK","Lệch "&amp;TEXT(H99-$G99,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J99" s="28" t="n"/>
@@ -21783,7 +21783,7 @@
         <v/>
       </c>
       <c r="I102" s="41">
-        <f>IF($A102="","",IF($G102=0,"chưa nhập FY target",IF(ROUND(H102-$G102,2)=0,"OK","Lệch "&amp;TEXT(H102-$G102,"#,##0"))))</f>
+        <f>IF($A$96="","",IF($G102=0,"chưa nhập FY target",IF(ROUND(H102-$G102,2)=0,"OK","Lệch "&amp;TEXT(H102-$G102,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J102" s="28" t="n"/>
@@ -22215,7 +22215,7 @@
         <v/>
       </c>
       <c r="I105" s="41">
-        <f>IF($A105="","",IF($G105=0,"chưa nhập FY target",IF(ROUND(H105-$G105,2)=0,"OK","Lệch "&amp;TEXT(H105-$G105,"#,##0"))))</f>
+        <f>IF($A$96="","",IF($G105=0,"chưa nhập FY target",IF(ROUND(H105-$G105,2)=0,"OK","Lệch "&amp;TEXT(H105-$G105,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J105" s="28" t="n"/>
@@ -22647,7 +22647,7 @@
         <v/>
       </c>
       <c r="I108" s="41">
-        <f>IF($A108="","",IF($G108=0,"chưa nhập FY target",IF(ROUND(H108-$G108,2)=0,"OK","Lệch "&amp;TEXT(H108-$G108,"#,##0"))))</f>
+        <f>IF($A$96="","",IF($G108=0,"chưa nhập FY target",IF(ROUND(H108-$G108,2)=0,"OK","Lệch "&amp;TEXT(H108-$G108,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J108" s="28" t="n"/>
@@ -23085,7 +23085,7 @@
         <v/>
       </c>
       <c r="I111" s="41">
-        <f>IF($A111="","",IF($G111=0,"chưa nhập FY target",IF(ROUND(H111-$G111,2)=0,"OK","Lệch "&amp;TEXT(H111-$G111,"#,##0"))))</f>
+        <f>IF($A$111="","",IF($G111=0,"chưa nhập FY target",IF(ROUND(H111-$G111,2)=0,"OK","Lệch "&amp;TEXT(H111-$G111,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J111" s="28" t="n"/>
@@ -23517,7 +23517,7 @@
         <v/>
       </c>
       <c r="I114" s="41">
-        <f>IF($A114="","",IF($G114=0,"chưa nhập FY target",IF(ROUND(H114-$G114,2)=0,"OK","Lệch "&amp;TEXT(H114-$G114,"#,##0"))))</f>
+        <f>IF($A$111="","",IF($G114=0,"chưa nhập FY target",IF(ROUND(H114-$G114,2)=0,"OK","Lệch "&amp;TEXT(H114-$G114,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J114" s="28" t="n"/>
@@ -23949,7 +23949,7 @@
         <v/>
       </c>
       <c r="I117" s="41">
-        <f>IF($A117="","",IF($G117=0,"chưa nhập FY target",IF(ROUND(H117-$G117,2)=0,"OK","Lệch "&amp;TEXT(H117-$G117,"#,##0"))))</f>
+        <f>IF($A$111="","",IF($G117=0,"chưa nhập FY target",IF(ROUND(H117-$G117,2)=0,"OK","Lệch "&amp;TEXT(H117-$G117,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J117" s="28" t="n"/>
@@ -24381,7 +24381,7 @@
         <v/>
       </c>
       <c r="I120" s="41">
-        <f>IF($A120="","",IF($G120=0,"chưa nhập FY target",IF(ROUND(H120-$G120,2)=0,"OK","Lệch "&amp;TEXT(H120-$G120,"#,##0"))))</f>
+        <f>IF($A$111="","",IF($G120=0,"chưa nhập FY target",IF(ROUND(H120-$G120,2)=0,"OK","Lệch "&amp;TEXT(H120-$G120,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J120" s="28" t="n"/>
@@ -24813,7 +24813,7 @@
         <v/>
       </c>
       <c r="I123" s="41">
-        <f>IF($A123="","",IF($G123=0,"chưa nhập FY target",IF(ROUND(H123-$G123,2)=0,"OK","Lệch "&amp;TEXT(H123-$G123,"#,##0"))))</f>
+        <f>IF($A$111="","",IF($G123=0,"chưa nhập FY target",IF(ROUND(H123-$G123,2)=0,"OK","Lệch "&amp;TEXT(H123-$G123,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J123" s="28" t="n"/>
@@ -25251,7 +25251,7 @@
         <v/>
       </c>
       <c r="I126" s="41">
-        <f>IF($A126="","",IF($G126=0,"chưa nhập FY target",IF(ROUND(H126-$G126,2)=0,"OK","Lệch "&amp;TEXT(H126-$G126,"#,##0"))))</f>
+        <f>IF($A$126="","",IF($G126=0,"chưa nhập FY target",IF(ROUND(H126-$G126,2)=0,"OK","Lệch "&amp;TEXT(H126-$G126,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J126" s="28" t="n"/>
@@ -25683,7 +25683,7 @@
         <v/>
       </c>
       <c r="I129" s="41">
-        <f>IF($A129="","",IF($G129=0,"chưa nhập FY target",IF(ROUND(H129-$G129,2)=0,"OK","Lệch "&amp;TEXT(H129-$G129,"#,##0"))))</f>
+        <f>IF($A$126="","",IF($G129=0,"chưa nhập FY target",IF(ROUND(H129-$G129,2)=0,"OK","Lệch "&amp;TEXT(H129-$G129,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J129" s="28" t="n"/>
@@ -26115,7 +26115,7 @@
         <v/>
       </c>
       <c r="I132" s="41">
-        <f>IF($A132="","",IF($G132=0,"chưa nhập FY target",IF(ROUND(H132-$G132,2)=0,"OK","Lệch "&amp;TEXT(H132-$G132,"#,##0"))))</f>
+        <f>IF($A$126="","",IF($G132=0,"chưa nhập FY target",IF(ROUND(H132-$G132,2)=0,"OK","Lệch "&amp;TEXT(H132-$G132,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J132" s="28" t="n"/>
@@ -26547,7 +26547,7 @@
         <v/>
       </c>
       <c r="I135" s="41">
-        <f>IF($A135="","",IF($G135=0,"chưa nhập FY target",IF(ROUND(H135-$G135,2)=0,"OK","Lệch "&amp;TEXT(H135-$G135,"#,##0"))))</f>
+        <f>IF($A$126="","",IF($G135=0,"chưa nhập FY target",IF(ROUND(H135-$G135,2)=0,"OK","Lệch "&amp;TEXT(H135-$G135,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J135" s="28" t="n"/>
@@ -26979,7 +26979,7 @@
         <v/>
       </c>
       <c r="I138" s="41">
-        <f>IF($A138="","",IF($G138=0,"chưa nhập FY target",IF(ROUND(H138-$G138,2)=0,"OK","Lệch "&amp;TEXT(H138-$G138,"#,##0"))))</f>
+        <f>IF($A$126="","",IF($G138=0,"chưa nhập FY target",IF(ROUND(H138-$G138,2)=0,"OK","Lệch "&amp;TEXT(H138-$G138,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J138" s="28" t="n"/>
@@ -27417,7 +27417,7 @@
         <v/>
       </c>
       <c r="I141" s="41">
-        <f>IF($A141="","",IF($G141=0,"chưa nhập FY target",IF(ROUND(H141-$G141,2)=0,"OK","Lệch "&amp;TEXT(H141-$G141,"#,##0"))))</f>
+        <f>IF($A$141="","",IF($G141=0,"chưa nhập FY target",IF(ROUND(H141-$G141,2)=0,"OK","Lệch "&amp;TEXT(H141-$G141,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J141" s="28" t="n"/>
@@ -27849,7 +27849,7 @@
         <v/>
       </c>
       <c r="I144" s="41">
-        <f>IF($A144="","",IF($G144=0,"chưa nhập FY target",IF(ROUND(H144-$G144,2)=0,"OK","Lệch "&amp;TEXT(H144-$G144,"#,##0"))))</f>
+        <f>IF($A$141="","",IF($G144=0,"chưa nhập FY target",IF(ROUND(H144-$G144,2)=0,"OK","Lệch "&amp;TEXT(H144-$G144,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J144" s="28" t="n"/>
@@ -28281,7 +28281,7 @@
         <v/>
       </c>
       <c r="I147" s="41">
-        <f>IF($A147="","",IF($G147=0,"chưa nhập FY target",IF(ROUND(H147-$G147,2)=0,"OK","Lệch "&amp;TEXT(H147-$G147,"#,##0"))))</f>
+        <f>IF($A$141="","",IF($G147=0,"chưa nhập FY target",IF(ROUND(H147-$G147,2)=0,"OK","Lệch "&amp;TEXT(H147-$G147,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J147" s="28" t="n"/>
@@ -28713,7 +28713,7 @@
         <v/>
       </c>
       <c r="I150" s="41">
-        <f>IF($A150="","",IF($G150=0,"chưa nhập FY target",IF(ROUND(H150-$G150,2)=0,"OK","Lệch "&amp;TEXT(H150-$G150,"#,##0"))))</f>
+        <f>IF($A$141="","",IF($G150=0,"chưa nhập FY target",IF(ROUND(H150-$G150,2)=0,"OK","Lệch "&amp;TEXT(H150-$G150,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J150" s="28" t="n"/>
@@ -29145,7 +29145,7 @@
         <v/>
       </c>
       <c r="I153" s="41">
-        <f>IF($A153="","",IF($G153=0,"chưa nhập FY target",IF(ROUND(H153-$G153,2)=0,"OK","Lệch "&amp;TEXT(H153-$G153,"#,##0"))))</f>
+        <f>IF($A$141="","",IF($G153=0,"chưa nhập FY target",IF(ROUND(H153-$G153,2)=0,"OK","Lệch "&amp;TEXT(H153-$G153,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J153" s="28" t="n"/>
@@ -29583,7 +29583,7 @@
         <v/>
       </c>
       <c r="I156" s="41">
-        <f>IF($A156="","",IF($G156=0,"chưa nhập FY target",IF(ROUND(H156-$G156,2)=0,"OK","Lệch "&amp;TEXT(H156-$G156,"#,##0"))))</f>
+        <f>IF($A$156="","",IF($G156=0,"chưa nhập FY target",IF(ROUND(H156-$G156,2)=0,"OK","Lệch "&amp;TEXT(H156-$G156,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J156" s="28" t="n"/>
@@ -30015,7 +30015,7 @@
         <v/>
       </c>
       <c r="I159" s="41">
-        <f>IF($A159="","",IF($G159=0,"chưa nhập FY target",IF(ROUND(H159-$G159,2)=0,"OK","Lệch "&amp;TEXT(H159-$G159,"#,##0"))))</f>
+        <f>IF($A$156="","",IF($G159=0,"chưa nhập FY target",IF(ROUND(H159-$G159,2)=0,"OK","Lệch "&amp;TEXT(H159-$G159,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J159" s="28" t="n"/>
@@ -30447,7 +30447,7 @@
         <v/>
       </c>
       <c r="I162" s="41">
-        <f>IF($A162="","",IF($G162=0,"chưa nhập FY target",IF(ROUND(H162-$G162,2)=0,"OK","Lệch "&amp;TEXT(H162-$G162,"#,##0"))))</f>
+        <f>IF($A$156="","",IF($G162=0,"chưa nhập FY target",IF(ROUND(H162-$G162,2)=0,"OK","Lệch "&amp;TEXT(H162-$G162,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J162" s="28" t="n"/>
@@ -30879,7 +30879,7 @@
         <v/>
       </c>
       <c r="I165" s="41">
-        <f>IF($A165="","",IF($G165=0,"chưa nhập FY target",IF(ROUND(H165-$G165,2)=0,"OK","Lệch "&amp;TEXT(H165-$G165,"#,##0"))))</f>
+        <f>IF($A$156="","",IF($G165=0,"chưa nhập FY target",IF(ROUND(H165-$G165,2)=0,"OK","Lệch "&amp;TEXT(H165-$G165,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J165" s="28" t="n"/>
@@ -31311,7 +31311,7 @@
         <v/>
       </c>
       <c r="I168" s="41">
-        <f>IF($A168="","",IF($G168=0,"chưa nhập FY target",IF(ROUND(H168-$G168,2)=0,"OK","Lệch "&amp;TEXT(H168-$G168,"#,##0"))))</f>
+        <f>IF($A$156="","",IF($G168=0,"chưa nhập FY target",IF(ROUND(H168-$G168,2)=0,"OK","Lệch "&amp;TEXT(H168-$G168,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J168" s="28" t="n"/>
@@ -31749,7 +31749,7 @@
         <v/>
       </c>
       <c r="I171" s="41">
-        <f>IF($A171="","",IF($G171=0,"chưa nhập FY target",IF(ROUND(H171-$G171,2)=0,"OK","Lệch "&amp;TEXT(H171-$G171,"#,##0"))))</f>
+        <f>IF($A$171="","",IF($G171=0,"chưa nhập FY target",IF(ROUND(H171-$G171,2)=0,"OK","Lệch "&amp;TEXT(H171-$G171,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J171" s="28" t="n"/>
@@ -32181,7 +32181,7 @@
         <v/>
       </c>
       <c r="I174" s="41">
-        <f>IF($A174="","",IF($G174=0,"chưa nhập FY target",IF(ROUND(H174-$G174,2)=0,"OK","Lệch "&amp;TEXT(H174-$G174,"#,##0"))))</f>
+        <f>IF($A$171="","",IF($G174=0,"chưa nhập FY target",IF(ROUND(H174-$G174,2)=0,"OK","Lệch "&amp;TEXT(H174-$G174,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J174" s="28" t="n"/>
@@ -32613,7 +32613,7 @@
         <v/>
       </c>
       <c r="I177" s="41">
-        <f>IF($A177="","",IF($G177=0,"chưa nhập FY target",IF(ROUND(H177-$G177,2)=0,"OK","Lệch "&amp;TEXT(H177-$G177,"#,##0"))))</f>
+        <f>IF($A$171="","",IF($G177=0,"chưa nhập FY target",IF(ROUND(H177-$G177,2)=0,"OK","Lệch "&amp;TEXT(H177-$G177,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J177" s="28" t="n"/>
@@ -33045,7 +33045,7 @@
         <v/>
       </c>
       <c r="I180" s="41">
-        <f>IF($A180="","",IF($G180=0,"chưa nhập FY target",IF(ROUND(H180-$G180,2)=0,"OK","Lệch "&amp;TEXT(H180-$G180,"#,##0"))))</f>
+        <f>IF($A$171="","",IF($G180=0,"chưa nhập FY target",IF(ROUND(H180-$G180,2)=0,"OK","Lệch "&amp;TEXT(H180-$G180,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J180" s="28" t="n"/>
@@ -33477,7 +33477,7 @@
         <v/>
       </c>
       <c r="I183" s="41">
-        <f>IF($A183="","",IF($G183=0,"chưa nhập FY target",IF(ROUND(H183-$G183,2)=0,"OK","Lệch "&amp;TEXT(H183-$G183,"#,##0"))))</f>
+        <f>IF($A$171="","",IF($G183=0,"chưa nhập FY target",IF(ROUND(H183-$G183,2)=0,"OK","Lệch "&amp;TEXT(H183-$G183,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J183" s="28" t="n"/>
@@ -33915,7 +33915,7 @@
         <v/>
       </c>
       <c r="I186" s="41">
-        <f>IF($A186="","",IF($G186=0,"chưa nhập FY target",IF(ROUND(H186-$G186,2)=0,"OK","Lệch "&amp;TEXT(H186-$G186,"#,##0"))))</f>
+        <f>IF($A$186="","",IF($G186=0,"chưa nhập FY target",IF(ROUND(H186-$G186,2)=0,"OK","Lệch "&amp;TEXT(H186-$G186,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J186" s="28" t="n"/>
@@ -34347,7 +34347,7 @@
         <v/>
       </c>
       <c r="I189" s="41">
-        <f>IF($A189="","",IF($G189=0,"chưa nhập FY target",IF(ROUND(H189-$G189,2)=0,"OK","Lệch "&amp;TEXT(H189-$G189,"#,##0"))))</f>
+        <f>IF($A$186="","",IF($G189=0,"chưa nhập FY target",IF(ROUND(H189-$G189,2)=0,"OK","Lệch "&amp;TEXT(H189-$G189,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J189" s="28" t="n"/>
@@ -34779,7 +34779,7 @@
         <v/>
       </c>
       <c r="I192" s="41">
-        <f>IF($A192="","",IF($G192=0,"chưa nhập FY target",IF(ROUND(H192-$G192,2)=0,"OK","Lệch "&amp;TEXT(H192-$G192,"#,##0"))))</f>
+        <f>IF($A$186="","",IF($G192=0,"chưa nhập FY target",IF(ROUND(H192-$G192,2)=0,"OK","Lệch "&amp;TEXT(H192-$G192,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J192" s="28" t="n"/>
@@ -35211,7 +35211,7 @@
         <v/>
       </c>
       <c r="I195" s="41">
-        <f>IF($A195="","",IF($G195=0,"chưa nhập FY target",IF(ROUND(H195-$G195,2)=0,"OK","Lệch "&amp;TEXT(H195-$G195,"#,##0"))))</f>
+        <f>IF($A$186="","",IF($G195=0,"chưa nhập FY target",IF(ROUND(H195-$G195,2)=0,"OK","Lệch "&amp;TEXT(H195-$G195,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J195" s="28" t="n"/>
@@ -35643,7 +35643,7 @@
         <v/>
       </c>
       <c r="I198" s="41">
-        <f>IF($A198="","",IF($G198=0,"chưa nhập FY target",IF(ROUND(H198-$G198,2)=0,"OK","Lệch "&amp;TEXT(H198-$G198,"#,##0"))))</f>
+        <f>IF($A$186="","",IF($G198=0,"chưa nhập FY target",IF(ROUND(H198-$G198,2)=0,"OK","Lệch "&amp;TEXT(H198-$G198,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J198" s="28" t="n"/>
@@ -36081,7 +36081,7 @@
         <v/>
       </c>
       <c r="I201" s="41">
-        <f>IF($A201="","",IF($G201=0,"chưa nhập FY target",IF(ROUND(H201-$G201,2)=0,"OK","Lệch "&amp;TEXT(H201-$G201,"#,##0"))))</f>
+        <f>IF($A$201="","",IF($G201=0,"chưa nhập FY target",IF(ROUND(H201-$G201,2)=0,"OK","Lệch "&amp;TEXT(H201-$G201,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J201" s="28" t="n"/>
@@ -36513,7 +36513,7 @@
         <v/>
       </c>
       <c r="I204" s="41">
-        <f>IF($A204="","",IF($G204=0,"chưa nhập FY target",IF(ROUND(H204-$G204,2)=0,"OK","Lệch "&amp;TEXT(H204-$G204,"#,##0"))))</f>
+        <f>IF($A$201="","",IF($G204=0,"chưa nhập FY target",IF(ROUND(H204-$G204,2)=0,"OK","Lệch "&amp;TEXT(H204-$G204,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J204" s="28" t="n"/>
@@ -36945,7 +36945,7 @@
         <v/>
       </c>
       <c r="I207" s="41">
-        <f>IF($A207="","",IF($G207=0,"chưa nhập FY target",IF(ROUND(H207-$G207,2)=0,"OK","Lệch "&amp;TEXT(H207-$G207,"#,##0"))))</f>
+        <f>IF($A$201="","",IF($G207=0,"chưa nhập FY target",IF(ROUND(H207-$G207,2)=0,"OK","Lệch "&amp;TEXT(H207-$G207,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J207" s="28" t="n"/>
@@ -37377,7 +37377,7 @@
         <v/>
       </c>
       <c r="I210" s="41">
-        <f>IF($A210="","",IF($G210=0,"chưa nhập FY target",IF(ROUND(H210-$G210,2)=0,"OK","Lệch "&amp;TEXT(H210-$G210,"#,##0"))))</f>
+        <f>IF($A$201="","",IF($G210=0,"chưa nhập FY target",IF(ROUND(H210-$G210,2)=0,"OK","Lệch "&amp;TEXT(H210-$G210,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J210" s="28" t="n"/>
@@ -37809,7 +37809,7 @@
         <v/>
       </c>
       <c r="I213" s="41">
-        <f>IF($A213="","",IF($G213=0,"chưa nhập FY target",IF(ROUND(H213-$G213,2)=0,"OK","Lệch "&amp;TEXT(H213-$G213,"#,##0"))))</f>
+        <f>IF($A$201="","",IF($G213=0,"chưa nhập FY target",IF(ROUND(H213-$G213,2)=0,"OK","Lệch "&amp;TEXT(H213-$G213,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J213" s="28" t="n"/>
@@ -38247,7 +38247,7 @@
         <v/>
       </c>
       <c r="I216" s="41">
-        <f>IF($A216="","",IF($G216=0,"chưa nhập FY target",IF(ROUND(H216-$G216,2)=0,"OK","Lệch "&amp;TEXT(H216-$G216,"#,##0"))))</f>
+        <f>IF($A$216="","",IF($G216=0,"chưa nhập FY target",IF(ROUND(H216-$G216,2)=0,"OK","Lệch "&amp;TEXT(H216-$G216,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J216" s="28" t="n"/>
@@ -38679,7 +38679,7 @@
         <v/>
       </c>
       <c r="I219" s="41">
-        <f>IF($A219="","",IF($G219=0,"chưa nhập FY target",IF(ROUND(H219-$G219,2)=0,"OK","Lệch "&amp;TEXT(H219-$G219,"#,##0"))))</f>
+        <f>IF($A$216="","",IF($G219=0,"chưa nhập FY target",IF(ROUND(H219-$G219,2)=0,"OK","Lệch "&amp;TEXT(H219-$G219,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J219" s="28" t="n"/>
@@ -39111,7 +39111,7 @@
         <v/>
       </c>
       <c r="I222" s="41">
-        <f>IF($A222="","",IF($G222=0,"chưa nhập FY target",IF(ROUND(H222-$G222,2)=0,"OK","Lệch "&amp;TEXT(H222-$G222,"#,##0"))))</f>
+        <f>IF($A$216="","",IF($G222=0,"chưa nhập FY target",IF(ROUND(H222-$G222,2)=0,"OK","Lệch "&amp;TEXT(H222-$G222,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J222" s="28" t="n"/>
@@ -39543,7 +39543,7 @@
         <v/>
       </c>
       <c r="I225" s="41">
-        <f>IF($A225="","",IF($G225=0,"chưa nhập FY target",IF(ROUND(H225-$G225,2)=0,"OK","Lệch "&amp;TEXT(H225-$G225,"#,##0"))))</f>
+        <f>IF($A$216="","",IF($G225=0,"chưa nhập FY target",IF(ROUND(H225-$G225,2)=0,"OK","Lệch "&amp;TEXT(H225-$G225,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J225" s="28" t="n"/>
@@ -39975,7 +39975,7 @@
         <v/>
       </c>
       <c r="I228" s="41">
-        <f>IF($A228="","",IF($G228=0,"chưa nhập FY target",IF(ROUND(H228-$G228,2)=0,"OK","Lệch "&amp;TEXT(H228-$G228,"#,##0"))))</f>
+        <f>IF($A$216="","",IF($G228=0,"chưa nhập FY target",IF(ROUND(H228-$G228,2)=0,"OK","Lệch "&amp;TEXT(H228-$G228,"#,##0"))))</f>
         <v/>
       </c>
       <c r="J228" s="28" t="n"/>
@@ -41070,7 +41070,7 @@
         <v/>
       </c>
       <c r="Y6" s="68">
-        <f>IF($A6="","",IF(F6&lt;=0,"No target",IF(X6&gt;=1,"On track",IF(X6&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A6="","",IF(1&gt;Setup!$C$5,"Chưa chốt",IF(F6&lt;=0,"No target",IF(X6&gt;=1,"On track",IF(X6&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z6" s="69">
@@ -41184,7 +41184,7 @@
         <v/>
       </c>
       <c r="Y7" s="68">
-        <f>IF($A7="","",IF(F7&lt;=0,"No target",IF(X7&gt;=1,"On track",IF(X7&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A7="","",IF(2&gt;Setup!$C$5,"Chưa chốt",IF(F7&lt;=0,"No target",IF(X7&gt;=1,"On track",IF(X7&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z7" s="69">
@@ -41298,7 +41298,7 @@
         <v/>
       </c>
       <c r="Y8" s="68">
-        <f>IF($A8="","",IF(F8&lt;=0,"No target",IF(X8&gt;=1,"On track",IF(X8&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A8="","",IF(3&gt;Setup!$C$5,"Chưa chốt",IF(F8&lt;=0,"No target",IF(X8&gt;=1,"On track",IF(X8&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z8" s="69">
@@ -41412,7 +41412,7 @@
         <v/>
       </c>
       <c r="Y9" s="68">
-        <f>IF($A9="","",IF(F9&lt;=0,"No target",IF(X9&gt;=1,"On track",IF(X9&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A9="","",IF(4&gt;Setup!$C$5,"Chưa chốt",IF(F9&lt;=0,"No target",IF(X9&gt;=1,"On track",IF(X9&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z9" s="69">
@@ -41526,7 +41526,7 @@
         <v/>
       </c>
       <c r="Y10" s="68">
-        <f>IF($A10="","",IF(F10&lt;=0,"No target",IF(X10&gt;=1,"On track",IF(X10&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A10="","",IF(1&gt;Setup!$C$5,"Chưa chốt",IF(F10&lt;=0,"No target",IF(X10&gt;=1,"On track",IF(X10&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z10" s="69">
@@ -41640,7 +41640,7 @@
         <v/>
       </c>
       <c r="Y11" s="68">
-        <f>IF($A11="","",IF(F11&lt;=0,"No target",IF(X11&gt;=1,"On track",IF(X11&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A11="","",IF(2&gt;Setup!$C$5,"Chưa chốt",IF(F11&lt;=0,"No target",IF(X11&gt;=1,"On track",IF(X11&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z11" s="69">
@@ -41754,7 +41754,7 @@
         <v/>
       </c>
       <c r="Y12" s="68">
-        <f>IF($A12="","",IF(F12&lt;=0,"No target",IF(X12&gt;=1,"On track",IF(X12&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A12="","",IF(3&gt;Setup!$C$5,"Chưa chốt",IF(F12&lt;=0,"No target",IF(X12&gt;=1,"On track",IF(X12&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z12" s="69">
@@ -41868,7 +41868,7 @@
         <v/>
       </c>
       <c r="Y13" s="68">
-        <f>IF($A13="","",IF(F13&lt;=0,"No target",IF(X13&gt;=1,"On track",IF(X13&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A13="","",IF(4&gt;Setup!$C$5,"Chưa chốt",IF(F13&lt;=0,"No target",IF(X13&gt;=1,"On track",IF(X13&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z13" s="69">
@@ -41982,7 +41982,7 @@
         <v/>
       </c>
       <c r="Y14" s="68">
-        <f>IF($A14="","",IF(F14&lt;=0,"No target",IF(X14&gt;=1,"On track",IF(X14&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A14="","",IF(1&gt;Setup!$C$5,"Chưa chốt",IF(F14&lt;=0,"No target",IF(X14&gt;=1,"On track",IF(X14&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z14" s="69">
@@ -42096,7 +42096,7 @@
         <v/>
       </c>
       <c r="Y15" s="68">
-        <f>IF($A15="","",IF(F15&lt;=0,"No target",IF(X15&gt;=1,"On track",IF(X15&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A15="","",IF(2&gt;Setup!$C$5,"Chưa chốt",IF(F15&lt;=0,"No target",IF(X15&gt;=1,"On track",IF(X15&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z15" s="69">
@@ -42210,7 +42210,7 @@
         <v/>
       </c>
       <c r="Y16" s="68">
-        <f>IF($A16="","",IF(F16&lt;=0,"No target",IF(X16&gt;=1,"On track",IF(X16&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A16="","",IF(3&gt;Setup!$C$5,"Chưa chốt",IF(F16&lt;=0,"No target",IF(X16&gt;=1,"On track",IF(X16&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z16" s="69">
@@ -42324,7 +42324,7 @@
         <v/>
       </c>
       <c r="Y17" s="68">
-        <f>IF($A17="","",IF(F17&lt;=0,"No target",IF(X17&gt;=1,"On track",IF(X17&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A17="","",IF(4&gt;Setup!$C$5,"Chưa chốt",IF(F17&lt;=0,"No target",IF(X17&gt;=1,"On track",IF(X17&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z17" s="69">
@@ -42438,7 +42438,7 @@
         <v/>
       </c>
       <c r="Y18" s="68">
-        <f>IF($A18="","",IF(F18&lt;=0,"No target",IF(X18&gt;=1,"On track",IF(X18&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A18="","",IF(1&gt;Setup!$C$5,"Chưa chốt",IF(F18&lt;=0,"No target",IF(X18&gt;=1,"On track",IF(X18&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z18" s="69">
@@ -42552,7 +42552,7 @@
         <v/>
       </c>
       <c r="Y19" s="68">
-        <f>IF($A19="","",IF(F19&lt;=0,"No target",IF(X19&gt;=1,"On track",IF(X19&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A19="","",IF(2&gt;Setup!$C$5,"Chưa chốt",IF(F19&lt;=0,"No target",IF(X19&gt;=1,"On track",IF(X19&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z19" s="69">
@@ -42666,7 +42666,7 @@
         <v/>
       </c>
       <c r="Y20" s="68">
-        <f>IF($A20="","",IF(F20&lt;=0,"No target",IF(X20&gt;=1,"On track",IF(X20&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A20="","",IF(3&gt;Setup!$C$5,"Chưa chốt",IF(F20&lt;=0,"No target",IF(X20&gt;=1,"On track",IF(X20&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z20" s="69">
@@ -42780,7 +42780,7 @@
         <v/>
       </c>
       <c r="Y21" s="68">
-        <f>IF($A21="","",IF(F21&lt;=0,"No target",IF(X21&gt;=1,"On track",IF(X21&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A21="","",IF(4&gt;Setup!$C$5,"Chưa chốt",IF(F21&lt;=0,"No target",IF(X21&gt;=1,"On track",IF(X21&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z21" s="69">
@@ -42894,7 +42894,7 @@
         <v/>
       </c>
       <c r="Y22" s="68">
-        <f>IF($A22="","",IF(F22&lt;=0,"No target",IF(X22&gt;=1,"On track",IF(X22&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A22="","",IF(1&gt;Setup!$C$5,"Chưa chốt",IF(F22&lt;=0,"No target",IF(X22&gt;=1,"On track",IF(X22&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z22" s="69">
@@ -43008,7 +43008,7 @@
         <v/>
       </c>
       <c r="Y23" s="68">
-        <f>IF($A23="","",IF(F23&lt;=0,"No target",IF(X23&gt;=1,"On track",IF(X23&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A23="","",IF(2&gt;Setup!$C$5,"Chưa chốt",IF(F23&lt;=0,"No target",IF(X23&gt;=1,"On track",IF(X23&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z23" s="69">
@@ -43122,7 +43122,7 @@
         <v/>
       </c>
       <c r="Y24" s="68">
-        <f>IF($A24="","",IF(F24&lt;=0,"No target",IF(X24&gt;=1,"On track",IF(X24&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A24="","",IF(3&gt;Setup!$C$5,"Chưa chốt",IF(F24&lt;=0,"No target",IF(X24&gt;=1,"On track",IF(X24&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z24" s="69">
@@ -43236,7 +43236,7 @@
         <v/>
       </c>
       <c r="Y25" s="68">
-        <f>IF($A25="","",IF(F25&lt;=0,"No target",IF(X25&gt;=1,"On track",IF(X25&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A25="","",IF(4&gt;Setup!$C$5,"Chưa chốt",IF(F25&lt;=0,"No target",IF(X25&gt;=1,"On track",IF(X25&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z25" s="69">
@@ -43350,7 +43350,7 @@
         <v/>
       </c>
       <c r="Y26" s="68">
-        <f>IF($A26="","",IF(F26&lt;=0,"No target",IF(X26&gt;=1,"On track",IF(X26&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A26="","",IF(1&gt;Setup!$C$5,"Chưa chốt",IF(F26&lt;=0,"No target",IF(X26&gt;=1,"On track",IF(X26&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z26" s="69">
@@ -43464,7 +43464,7 @@
         <v/>
       </c>
       <c r="Y27" s="68">
-        <f>IF($A27="","",IF(F27&lt;=0,"No target",IF(X27&gt;=1,"On track",IF(X27&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A27="","",IF(2&gt;Setup!$C$5,"Chưa chốt",IF(F27&lt;=0,"No target",IF(X27&gt;=1,"On track",IF(X27&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z27" s="69">
@@ -43578,7 +43578,7 @@
         <v/>
       </c>
       <c r="Y28" s="68">
-        <f>IF($A28="","",IF(F28&lt;=0,"No target",IF(X28&gt;=1,"On track",IF(X28&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A28="","",IF(3&gt;Setup!$C$5,"Chưa chốt",IF(F28&lt;=0,"No target",IF(X28&gt;=1,"On track",IF(X28&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z28" s="69">
@@ -43692,7 +43692,7 @@
         <v/>
       </c>
       <c r="Y29" s="68">
-        <f>IF($A29="","",IF(F29&lt;=0,"No target",IF(X29&gt;=1,"On track",IF(X29&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A29="","",IF(4&gt;Setup!$C$5,"Chưa chốt",IF(F29&lt;=0,"No target",IF(X29&gt;=1,"On track",IF(X29&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z29" s="69">
@@ -43806,7 +43806,7 @@
         <v/>
       </c>
       <c r="Y30" s="68">
-        <f>IF($A30="","",IF(F30&lt;=0,"No target",IF(X30&gt;=1,"On track",IF(X30&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A30="","",IF(1&gt;Setup!$C$5,"Chưa chốt",IF(F30&lt;=0,"No target",IF(X30&gt;=1,"On track",IF(X30&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z30" s="69">
@@ -43920,7 +43920,7 @@
         <v/>
       </c>
       <c r="Y31" s="68">
-        <f>IF($A31="","",IF(F31&lt;=0,"No target",IF(X31&gt;=1,"On track",IF(X31&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A31="","",IF(2&gt;Setup!$C$5,"Chưa chốt",IF(F31&lt;=0,"No target",IF(X31&gt;=1,"On track",IF(X31&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z31" s="69">
@@ -44034,7 +44034,7 @@
         <v/>
       </c>
       <c r="Y32" s="68">
-        <f>IF($A32="","",IF(F32&lt;=0,"No target",IF(X32&gt;=1,"On track",IF(X32&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A32="","",IF(3&gt;Setup!$C$5,"Chưa chốt",IF(F32&lt;=0,"No target",IF(X32&gt;=1,"On track",IF(X32&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z32" s="69">
@@ -44148,7 +44148,7 @@
         <v/>
       </c>
       <c r="Y33" s="68">
-        <f>IF($A33="","",IF(F33&lt;=0,"No target",IF(X33&gt;=1,"On track",IF(X33&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A33="","",IF(4&gt;Setup!$C$5,"Chưa chốt",IF(F33&lt;=0,"No target",IF(X33&gt;=1,"On track",IF(X33&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z33" s="69">
@@ -44262,7 +44262,7 @@
         <v/>
       </c>
       <c r="Y34" s="68">
-        <f>IF($A34="","",IF(F34&lt;=0,"No target",IF(X34&gt;=1,"On track",IF(X34&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A34="","",IF(1&gt;Setup!$C$5,"Chưa chốt",IF(F34&lt;=0,"No target",IF(X34&gt;=1,"On track",IF(X34&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z34" s="69">
@@ -44376,7 +44376,7 @@
         <v/>
       </c>
       <c r="Y35" s="68">
-        <f>IF($A35="","",IF(F35&lt;=0,"No target",IF(X35&gt;=1,"On track",IF(X35&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A35="","",IF(2&gt;Setup!$C$5,"Chưa chốt",IF(F35&lt;=0,"No target",IF(X35&gt;=1,"On track",IF(X35&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z35" s="69">
@@ -44490,7 +44490,7 @@
         <v/>
       </c>
       <c r="Y36" s="68">
-        <f>IF($A36="","",IF(F36&lt;=0,"No target",IF(X36&gt;=1,"On track",IF(X36&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A36="","",IF(3&gt;Setup!$C$5,"Chưa chốt",IF(F36&lt;=0,"No target",IF(X36&gt;=1,"On track",IF(X36&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z36" s="69">
@@ -44604,7 +44604,7 @@
         <v/>
       </c>
       <c r="Y37" s="68">
-        <f>IF($A37="","",IF(F37&lt;=0,"No target",IF(X37&gt;=1,"On track",IF(X37&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A37="","",IF(4&gt;Setup!$C$5,"Chưa chốt",IF(F37&lt;=0,"No target",IF(X37&gt;=1,"On track",IF(X37&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z37" s="69">
@@ -44718,7 +44718,7 @@
         <v/>
       </c>
       <c r="Y38" s="68">
-        <f>IF($A38="","",IF(F38&lt;=0,"No target",IF(X38&gt;=1,"On track",IF(X38&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A38="","",IF(1&gt;Setup!$C$5,"Chưa chốt",IF(F38&lt;=0,"No target",IF(X38&gt;=1,"On track",IF(X38&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z38" s="69">
@@ -44832,7 +44832,7 @@
         <v/>
       </c>
       <c r="Y39" s="68">
-        <f>IF($A39="","",IF(F39&lt;=0,"No target",IF(X39&gt;=1,"On track",IF(X39&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A39="","",IF(2&gt;Setup!$C$5,"Chưa chốt",IF(F39&lt;=0,"No target",IF(X39&gt;=1,"On track",IF(X39&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z39" s="69">
@@ -44946,7 +44946,7 @@
         <v/>
       </c>
       <c r="Y40" s="68">
-        <f>IF($A40="","",IF(F40&lt;=0,"No target",IF(X40&gt;=1,"On track",IF(X40&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A40="","",IF(3&gt;Setup!$C$5,"Chưa chốt",IF(F40&lt;=0,"No target",IF(X40&gt;=1,"On track",IF(X40&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z40" s="69">
@@ -45060,7 +45060,7 @@
         <v/>
       </c>
       <c r="Y41" s="68">
-        <f>IF($A41="","",IF(F41&lt;=0,"No target",IF(X41&gt;=1,"On track",IF(X41&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A41="","",IF(4&gt;Setup!$C$5,"Chưa chốt",IF(F41&lt;=0,"No target",IF(X41&gt;=1,"On track",IF(X41&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z41" s="69">
@@ -45174,7 +45174,7 @@
         <v/>
       </c>
       <c r="Y42" s="68">
-        <f>IF($A42="","",IF(F42&lt;=0,"No target",IF(X42&gt;=1,"On track",IF(X42&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A42="","",IF(1&gt;Setup!$C$5,"Chưa chốt",IF(F42&lt;=0,"No target",IF(X42&gt;=1,"On track",IF(X42&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z42" s="69">
@@ -45288,7 +45288,7 @@
         <v/>
       </c>
       <c r="Y43" s="68">
-        <f>IF($A43="","",IF(F43&lt;=0,"No target",IF(X43&gt;=1,"On track",IF(X43&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A43="","",IF(2&gt;Setup!$C$5,"Chưa chốt",IF(F43&lt;=0,"No target",IF(X43&gt;=1,"On track",IF(X43&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z43" s="69">
@@ -45402,7 +45402,7 @@
         <v/>
       </c>
       <c r="Y44" s="68">
-        <f>IF($A44="","",IF(F44&lt;=0,"No target",IF(X44&gt;=1,"On track",IF(X44&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A44="","",IF(3&gt;Setup!$C$5,"Chưa chốt",IF(F44&lt;=0,"No target",IF(X44&gt;=1,"On track",IF(X44&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z44" s="69">
@@ -45516,7 +45516,7 @@
         <v/>
       </c>
       <c r="Y45" s="68">
-        <f>IF($A45="","",IF(F45&lt;=0,"No target",IF(X45&gt;=1,"On track",IF(X45&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A45="","",IF(4&gt;Setup!$C$5,"Chưa chốt",IF(F45&lt;=0,"No target",IF(X45&gt;=1,"On track",IF(X45&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z45" s="69">
@@ -45630,7 +45630,7 @@
         <v/>
       </c>
       <c r="Y46" s="68">
-        <f>IF($A46="","",IF(F46&lt;=0,"No target",IF(X46&gt;=1,"On track",IF(X46&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A46="","",IF(1&gt;Setup!$C$5,"Chưa chốt",IF(F46&lt;=0,"No target",IF(X46&gt;=1,"On track",IF(X46&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z46" s="69">
@@ -45744,7 +45744,7 @@
         <v/>
       </c>
       <c r="Y47" s="68">
-        <f>IF($A47="","",IF(F47&lt;=0,"No target",IF(X47&gt;=1,"On track",IF(X47&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A47="","",IF(2&gt;Setup!$C$5,"Chưa chốt",IF(F47&lt;=0,"No target",IF(X47&gt;=1,"On track",IF(X47&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z47" s="69">
@@ -45858,7 +45858,7 @@
         <v/>
       </c>
       <c r="Y48" s="68">
-        <f>IF($A48="","",IF(F48&lt;=0,"No target",IF(X48&gt;=1,"On track",IF(X48&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A48="","",IF(3&gt;Setup!$C$5,"Chưa chốt",IF(F48&lt;=0,"No target",IF(X48&gt;=1,"On track",IF(X48&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z48" s="69">
@@ -45972,7 +45972,7 @@
         <v/>
       </c>
       <c r="Y49" s="68">
-        <f>IF($A49="","",IF(F49&lt;=0,"No target",IF(X49&gt;=1,"On track",IF(X49&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A49="","",IF(4&gt;Setup!$C$5,"Chưa chốt",IF(F49&lt;=0,"No target",IF(X49&gt;=1,"On track",IF(X49&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z49" s="69">
@@ -46086,7 +46086,7 @@
         <v/>
       </c>
       <c r="Y50" s="68">
-        <f>IF($A50="","",IF(F50&lt;=0,"No target",IF(X50&gt;=1,"On track",IF(X50&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A50="","",IF(1&gt;Setup!$C$5,"Chưa chốt",IF(F50&lt;=0,"No target",IF(X50&gt;=1,"On track",IF(X50&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z50" s="69">
@@ -46200,7 +46200,7 @@
         <v/>
       </c>
       <c r="Y51" s="68">
-        <f>IF($A51="","",IF(F51&lt;=0,"No target",IF(X51&gt;=1,"On track",IF(X51&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A51="","",IF(2&gt;Setup!$C$5,"Chưa chốt",IF(F51&lt;=0,"No target",IF(X51&gt;=1,"On track",IF(X51&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z51" s="69">
@@ -46314,7 +46314,7 @@
         <v/>
       </c>
       <c r="Y52" s="68">
-        <f>IF($A52="","",IF(F52&lt;=0,"No target",IF(X52&gt;=1,"On track",IF(X52&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A52="","",IF(3&gt;Setup!$C$5,"Chưa chốt",IF(F52&lt;=0,"No target",IF(X52&gt;=1,"On track",IF(X52&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z52" s="69">
@@ -46428,7 +46428,7 @@
         <v/>
       </c>
       <c r="Y53" s="68">
-        <f>IF($A53="","",IF(F53&lt;=0,"No target",IF(X53&gt;=1,"On track",IF(X53&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A53="","",IF(4&gt;Setup!$C$5,"Chưa chốt",IF(F53&lt;=0,"No target",IF(X53&gt;=1,"On track",IF(X53&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z53" s="69">
@@ -46542,7 +46542,7 @@
         <v/>
       </c>
       <c r="Y54" s="68">
-        <f>IF($A54="","",IF(F54&lt;=0,"No target",IF(X54&gt;=1,"On track",IF(X54&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A54="","",IF(1&gt;Setup!$C$5,"Chưa chốt",IF(F54&lt;=0,"No target",IF(X54&gt;=1,"On track",IF(X54&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z54" s="69">
@@ -46656,7 +46656,7 @@
         <v/>
       </c>
       <c r="Y55" s="68">
-        <f>IF($A55="","",IF(F55&lt;=0,"No target",IF(X55&gt;=1,"On track",IF(X55&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A55="","",IF(2&gt;Setup!$C$5,"Chưa chốt",IF(F55&lt;=0,"No target",IF(X55&gt;=1,"On track",IF(X55&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z55" s="69">
@@ -46770,7 +46770,7 @@
         <v/>
       </c>
       <c r="Y56" s="68">
-        <f>IF($A56="","",IF(F56&lt;=0,"No target",IF(X56&gt;=1,"On track",IF(X56&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A56="","",IF(3&gt;Setup!$C$5,"Chưa chốt",IF(F56&lt;=0,"No target",IF(X56&gt;=1,"On track",IF(X56&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z56" s="69">
@@ -46884,7 +46884,7 @@
         <v/>
       </c>
       <c r="Y57" s="68">
-        <f>IF($A57="","",IF(F57&lt;=0,"No target",IF(X57&gt;=1,"On track",IF(X57&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A57="","",IF(4&gt;Setup!$C$5,"Chưa chốt",IF(F57&lt;=0,"No target",IF(X57&gt;=1,"On track",IF(X57&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z57" s="69">
@@ -46998,7 +46998,7 @@
         <v/>
       </c>
       <c r="Y58" s="68">
-        <f>IF($A58="","",IF(F58&lt;=0,"No target",IF(X58&gt;=1,"On track",IF(X58&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A58="","",IF(1&gt;Setup!$C$5,"Chưa chốt",IF(F58&lt;=0,"No target",IF(X58&gt;=1,"On track",IF(X58&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z58" s="69">
@@ -47112,7 +47112,7 @@
         <v/>
       </c>
       <c r="Y59" s="68">
-        <f>IF($A59="","",IF(F59&lt;=0,"No target",IF(X59&gt;=1,"On track",IF(X59&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A59="","",IF(2&gt;Setup!$C$5,"Chưa chốt",IF(F59&lt;=0,"No target",IF(X59&gt;=1,"On track",IF(X59&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z59" s="69">
@@ -47226,7 +47226,7 @@
         <v/>
       </c>
       <c r="Y60" s="68">
-        <f>IF($A60="","",IF(F60&lt;=0,"No target",IF(X60&gt;=1,"On track",IF(X60&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A60="","",IF(3&gt;Setup!$C$5,"Chưa chốt",IF(F60&lt;=0,"No target",IF(X60&gt;=1,"On track",IF(X60&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z60" s="69">
@@ -47340,7 +47340,7 @@
         <v/>
       </c>
       <c r="Y61" s="68">
-        <f>IF($A61="","",IF(F61&lt;=0,"No target",IF(X61&gt;=1,"On track",IF(X61&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A61="","",IF(4&gt;Setup!$C$5,"Chưa chốt",IF(F61&lt;=0,"No target",IF(X61&gt;=1,"On track",IF(X61&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z61" s="69">
@@ -47454,7 +47454,7 @@
         <v/>
       </c>
       <c r="Y62" s="68">
-        <f>IF($A62="","",IF(F62&lt;=0,"No target",IF(X62&gt;=1,"On track",IF(X62&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A62="","",IF(1&gt;Setup!$C$5,"Chưa chốt",IF(F62&lt;=0,"No target",IF(X62&gt;=1,"On track",IF(X62&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z62" s="69">
@@ -47568,7 +47568,7 @@
         <v/>
       </c>
       <c r="Y63" s="68">
-        <f>IF($A63="","",IF(F63&lt;=0,"No target",IF(X63&gt;=1,"On track",IF(X63&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A63="","",IF(2&gt;Setup!$C$5,"Chưa chốt",IF(F63&lt;=0,"No target",IF(X63&gt;=1,"On track",IF(X63&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z63" s="69">
@@ -47682,7 +47682,7 @@
         <v/>
       </c>
       <c r="Y64" s="68">
-        <f>IF($A64="","",IF(F64&lt;=0,"No target",IF(X64&gt;=1,"On track",IF(X64&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A64="","",IF(3&gt;Setup!$C$5,"Chưa chốt",IF(F64&lt;=0,"No target",IF(X64&gt;=1,"On track",IF(X64&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z64" s="69">
@@ -47796,7 +47796,7 @@
         <v/>
       </c>
       <c r="Y65" s="68">
-        <f>IF($A65="","",IF(F65&lt;=0,"No target",IF(X65&gt;=1,"On track",IF(X65&gt;=0.8,"Watch","Behind"))))</f>
+        <f>IF($A65="","",IF(4&gt;Setup!$C$5,"Chưa chốt",IF(F65&lt;=0,"No target",IF(X65&gt;=1,"On track",IF(X65&gt;=0.8,"Watch","Behind")))))</f>
         <v/>
       </c>
       <c r="Z65" s="69">
@@ -48307,7 +48307,7 @@
       </c>
       <c r="U5" s="12" t="inlineStr">
         <is>
-          <t>Total Lead FY</t>
+          <t>Total Lead (đến quý chốt)</t>
         </is>
       </c>
       <c r="V5" s="56" t="inlineStr">
@@ -48327,7 +48327,7 @@
       </c>
       <c r="Y5" s="57" t="inlineStr">
         <is>
-          <t>TOTAL FY payout</t>
+          <t>TOTAL payout (đến quý chốt)</t>
         </is>
       </c>
       <c r="Z5" s="57" t="inlineStr">
@@ -48387,19 +48387,19 @@
         <v/>
       </c>
       <c r="M6" s="63">
-        <f>$H6*1/4*I6</f>
+        <f>IF(1&gt;Setup!$C$5,0,$G6*1/4*I6)</f>
         <v/>
       </c>
       <c r="N6" s="63">
-        <f>$H6*2/4*J6</f>
+        <f>IF(2&gt;Setup!$C$5,0,$G6*2/4*J6)</f>
         <v/>
       </c>
       <c r="O6" s="63">
-        <f>$H6*3/4*K6</f>
+        <f>IF(3&gt;Setup!$C$5,0,$G6*3/4*K6)</f>
         <v/>
       </c>
       <c r="P6" s="63">
-        <f>$H6*4/4*L6</f>
+        <f>IF(4&gt;Setup!$C$5,0,$G6*4/4*L6)</f>
         <v/>
       </c>
       <c r="Q6" s="83">
@@ -48431,7 +48431,7 @@
         <v/>
       </c>
       <c r="X6" s="84">
-        <f>$I6*W6</f>
+        <f>IF(Setup!$C$5&lt;4,0,$H6*W6)</f>
         <v/>
       </c>
       <c r="Y6" s="85">
@@ -48493,19 +48493,19 @@
         <v/>
       </c>
       <c r="M7" s="63">
-        <f>$H7*1/4*I7</f>
+        <f>IF(1&gt;Setup!$C$5,0,$G7*1/4*I7)</f>
         <v/>
       </c>
       <c r="N7" s="63">
-        <f>$H7*2/4*J7</f>
+        <f>IF(2&gt;Setup!$C$5,0,$G7*2/4*J7)</f>
         <v/>
       </c>
       <c r="O7" s="63">
-        <f>$H7*3/4*K7</f>
+        <f>IF(3&gt;Setup!$C$5,0,$G7*3/4*K7)</f>
         <v/>
       </c>
       <c r="P7" s="63">
-        <f>$H7*4/4*L7</f>
+        <f>IF(4&gt;Setup!$C$5,0,$G7*4/4*L7)</f>
         <v/>
       </c>
       <c r="Q7" s="83">
@@ -48537,7 +48537,7 @@
         <v/>
       </c>
       <c r="X7" s="84">
-        <f>$I7*W7</f>
+        <f>IF(Setup!$C$5&lt;4,0,$H7*W7)</f>
         <v/>
       </c>
       <c r="Y7" s="85">
@@ -48599,19 +48599,19 @@
         <v/>
       </c>
       <c r="M8" s="63">
-        <f>$H8*1/4*I8</f>
+        <f>IF(1&gt;Setup!$C$5,0,$G8*1/4*I8)</f>
         <v/>
       </c>
       <c r="N8" s="63">
-        <f>$H8*2/4*J8</f>
+        <f>IF(2&gt;Setup!$C$5,0,$G8*2/4*J8)</f>
         <v/>
       </c>
       <c r="O8" s="63">
-        <f>$H8*3/4*K8</f>
+        <f>IF(3&gt;Setup!$C$5,0,$G8*3/4*K8)</f>
         <v/>
       </c>
       <c r="P8" s="63">
-        <f>$H8*4/4*L8</f>
+        <f>IF(4&gt;Setup!$C$5,0,$G8*4/4*L8)</f>
         <v/>
       </c>
       <c r="Q8" s="83">
@@ -48643,7 +48643,7 @@
         <v/>
       </c>
       <c r="X8" s="84">
-        <f>$I8*W8</f>
+        <f>IF(Setup!$C$5&lt;4,0,$H8*W8)</f>
         <v/>
       </c>
       <c r="Y8" s="85">
@@ -48705,19 +48705,19 @@
         <v/>
       </c>
       <c r="M9" s="63">
-        <f>$H9*1/4*I9</f>
+        <f>IF(1&gt;Setup!$C$5,0,$G9*1/4*I9)</f>
         <v/>
       </c>
       <c r="N9" s="63">
-        <f>$H9*2/4*J9</f>
+        <f>IF(2&gt;Setup!$C$5,0,$G9*2/4*J9)</f>
         <v/>
       </c>
       <c r="O9" s="63">
-        <f>$H9*3/4*K9</f>
+        <f>IF(3&gt;Setup!$C$5,0,$G9*3/4*K9)</f>
         <v/>
       </c>
       <c r="P9" s="63">
-        <f>$H9*4/4*L9</f>
+        <f>IF(4&gt;Setup!$C$5,0,$G9*4/4*L9)</f>
         <v/>
       </c>
       <c r="Q9" s="83">
@@ -48749,7 +48749,7 @@
         <v/>
       </c>
       <c r="X9" s="84">
-        <f>$I9*W9</f>
+        <f>IF(Setup!$C$5&lt;4,0,$H9*W9)</f>
         <v/>
       </c>
       <c r="Y9" s="85">
@@ -48811,19 +48811,19 @@
         <v/>
       </c>
       <c r="M10" s="63">
-        <f>$H10*1/4*I10</f>
+        <f>IF(1&gt;Setup!$C$5,0,$G10*1/4*I10)</f>
         <v/>
       </c>
       <c r="N10" s="63">
-        <f>$H10*2/4*J10</f>
+        <f>IF(2&gt;Setup!$C$5,0,$G10*2/4*J10)</f>
         <v/>
       </c>
       <c r="O10" s="63">
-        <f>$H10*3/4*K10</f>
+        <f>IF(3&gt;Setup!$C$5,0,$G10*3/4*K10)</f>
         <v/>
       </c>
       <c r="P10" s="63">
-        <f>$H10*4/4*L10</f>
+        <f>IF(4&gt;Setup!$C$5,0,$G10*4/4*L10)</f>
         <v/>
       </c>
       <c r="Q10" s="83">
@@ -48855,7 +48855,7 @@
         <v/>
       </c>
       <c r="X10" s="84">
-        <f>$I10*W10</f>
+        <f>IF(Setup!$C$5&lt;4,0,$H10*W10)</f>
         <v/>
       </c>
       <c r="Y10" s="85">
@@ -48917,19 +48917,19 @@
         <v/>
       </c>
       <c r="M11" s="63">
-        <f>$H11*1/4*I11</f>
+        <f>IF(1&gt;Setup!$C$5,0,$G11*1/4*I11)</f>
         <v/>
       </c>
       <c r="N11" s="63">
-        <f>$H11*2/4*J11</f>
+        <f>IF(2&gt;Setup!$C$5,0,$G11*2/4*J11)</f>
         <v/>
       </c>
       <c r="O11" s="63">
-        <f>$H11*3/4*K11</f>
+        <f>IF(3&gt;Setup!$C$5,0,$G11*3/4*K11)</f>
         <v/>
       </c>
       <c r="P11" s="63">
-        <f>$H11*4/4*L11</f>
+        <f>IF(4&gt;Setup!$C$5,0,$G11*4/4*L11)</f>
         <v/>
       </c>
       <c r="Q11" s="83">
@@ -48961,7 +48961,7 @@
         <v/>
       </c>
       <c r="X11" s="84">
-        <f>$I11*W11</f>
+        <f>IF(Setup!$C$5&lt;4,0,$H11*W11)</f>
         <v/>
       </c>
       <c r="Y11" s="85">
@@ -49023,19 +49023,19 @@
         <v/>
       </c>
       <c r="M12" s="63">
-        <f>$H12*1/4*I12</f>
+        <f>IF(1&gt;Setup!$C$5,0,$G12*1/4*I12)</f>
         <v/>
       </c>
       <c r="N12" s="63">
-        <f>$H12*2/4*J12</f>
+        <f>IF(2&gt;Setup!$C$5,0,$G12*2/4*J12)</f>
         <v/>
       </c>
       <c r="O12" s="63">
-        <f>$H12*3/4*K12</f>
+        <f>IF(3&gt;Setup!$C$5,0,$G12*3/4*K12)</f>
         <v/>
       </c>
       <c r="P12" s="63">
-        <f>$H12*4/4*L12</f>
+        <f>IF(4&gt;Setup!$C$5,0,$G12*4/4*L12)</f>
         <v/>
       </c>
       <c r="Q12" s="83">
@@ -49067,7 +49067,7 @@
         <v/>
       </c>
       <c r="X12" s="84">
-        <f>$I12*W12</f>
+        <f>IF(Setup!$C$5&lt;4,0,$H12*W12)</f>
         <v/>
       </c>
       <c r="Y12" s="85">
@@ -49129,19 +49129,19 @@
         <v/>
       </c>
       <c r="M13" s="63">
-        <f>$H13*1/4*I13</f>
+        <f>IF(1&gt;Setup!$C$5,0,$G13*1/4*I13)</f>
         <v/>
       </c>
       <c r="N13" s="63">
-        <f>$H13*2/4*J13</f>
+        <f>IF(2&gt;Setup!$C$5,0,$G13*2/4*J13)</f>
         <v/>
       </c>
       <c r="O13" s="63">
-        <f>$H13*3/4*K13</f>
+        <f>IF(3&gt;Setup!$C$5,0,$G13*3/4*K13)</f>
         <v/>
       </c>
       <c r="P13" s="63">
-        <f>$H13*4/4*L13</f>
+        <f>IF(4&gt;Setup!$C$5,0,$G13*4/4*L13)</f>
         <v/>
       </c>
       <c r="Q13" s="83">
@@ -49173,7 +49173,7 @@
         <v/>
       </c>
       <c r="X13" s="84">
-        <f>$I13*W13</f>
+        <f>IF(Setup!$C$5&lt;4,0,$H13*W13)</f>
         <v/>
       </c>
       <c r="Y13" s="85">
@@ -49235,19 +49235,19 @@
         <v/>
       </c>
       <c r="M14" s="63">
-        <f>$H14*1/4*I14</f>
+        <f>IF(1&gt;Setup!$C$5,0,$G14*1/4*I14)</f>
         <v/>
       </c>
       <c r="N14" s="63">
-        <f>$H14*2/4*J14</f>
+        <f>IF(2&gt;Setup!$C$5,0,$G14*2/4*J14)</f>
         <v/>
       </c>
       <c r="O14" s="63">
-        <f>$H14*3/4*K14</f>
+        <f>IF(3&gt;Setup!$C$5,0,$G14*3/4*K14)</f>
         <v/>
       </c>
       <c r="P14" s="63">
-        <f>$H14*4/4*L14</f>
+        <f>IF(4&gt;Setup!$C$5,0,$G14*4/4*L14)</f>
         <v/>
       </c>
       <c r="Q14" s="83">
@@ -49279,7 +49279,7 @@
         <v/>
       </c>
       <c r="X14" s="84">
-        <f>$I14*W14</f>
+        <f>IF(Setup!$C$5&lt;4,0,$H14*W14)</f>
         <v/>
       </c>
       <c r="Y14" s="85">
@@ -49341,19 +49341,19 @@
         <v/>
       </c>
       <c r="M15" s="63">
-        <f>$H15*1/4*I15</f>
+        <f>IF(1&gt;Setup!$C$5,0,$G15*1/4*I15)</f>
         <v/>
       </c>
       <c r="N15" s="63">
-        <f>$H15*2/4*J15</f>
+        <f>IF(2&gt;Setup!$C$5,0,$G15*2/4*J15)</f>
         <v/>
       </c>
       <c r="O15" s="63">
-        <f>$H15*3/4*K15</f>
+        <f>IF(3&gt;Setup!$C$5,0,$G15*3/4*K15)</f>
         <v/>
       </c>
       <c r="P15" s="63">
-        <f>$H15*4/4*L15</f>
+        <f>IF(4&gt;Setup!$C$5,0,$G15*4/4*L15)</f>
         <v/>
       </c>
       <c r="Q15" s="83">
@@ -49385,7 +49385,7 @@
         <v/>
       </c>
       <c r="X15" s="84">
-        <f>$I15*W15</f>
+        <f>IF(Setup!$C$5&lt;4,0,$H15*W15)</f>
         <v/>
       </c>
       <c r="Y15" s="85">
@@ -49447,19 +49447,19 @@
         <v/>
       </c>
       <c r="M16" s="63">
-        <f>$H16*1/4*I16</f>
+        <f>IF(1&gt;Setup!$C$5,0,$G16*1/4*I16)</f>
         <v/>
       </c>
       <c r="N16" s="63">
-        <f>$H16*2/4*J16</f>
+        <f>IF(2&gt;Setup!$C$5,0,$G16*2/4*J16)</f>
         <v/>
       </c>
       <c r="O16" s="63">
-        <f>$H16*3/4*K16</f>
+        <f>IF(3&gt;Setup!$C$5,0,$G16*3/4*K16)</f>
         <v/>
       </c>
       <c r="P16" s="63">
-        <f>$H16*4/4*L16</f>
+        <f>IF(4&gt;Setup!$C$5,0,$G16*4/4*L16)</f>
         <v/>
       </c>
       <c r="Q16" s="83">
@@ -49491,7 +49491,7 @@
         <v/>
       </c>
       <c r="X16" s="84">
-        <f>$I16*W16</f>
+        <f>IF(Setup!$C$5&lt;4,0,$H16*W16)</f>
         <v/>
       </c>
       <c r="Y16" s="85">
@@ -49553,19 +49553,19 @@
         <v/>
       </c>
       <c r="M17" s="63">
-        <f>$H17*1/4*I17</f>
+        <f>IF(1&gt;Setup!$C$5,0,$G17*1/4*I17)</f>
         <v/>
       </c>
       <c r="N17" s="63">
-        <f>$H17*2/4*J17</f>
+        <f>IF(2&gt;Setup!$C$5,0,$G17*2/4*J17)</f>
         <v/>
       </c>
       <c r="O17" s="63">
-        <f>$H17*3/4*K17</f>
+        <f>IF(3&gt;Setup!$C$5,0,$G17*3/4*K17)</f>
         <v/>
       </c>
       <c r="P17" s="63">
-        <f>$H17*4/4*L17</f>
+        <f>IF(4&gt;Setup!$C$5,0,$G17*4/4*L17)</f>
         <v/>
       </c>
       <c r="Q17" s="83">
@@ -49597,7 +49597,7 @@
         <v/>
       </c>
       <c r="X17" s="84">
-        <f>$I17*W17</f>
+        <f>IF(Setup!$C$5&lt;4,0,$H17*W17)</f>
         <v/>
       </c>
       <c r="Y17" s="85">
@@ -49659,19 +49659,19 @@
         <v/>
       </c>
       <c r="M18" s="63">
-        <f>$H18*1/4*I18</f>
+        <f>IF(1&gt;Setup!$C$5,0,$G18*1/4*I18)</f>
         <v/>
       </c>
       <c r="N18" s="63">
-        <f>$H18*2/4*J18</f>
+        <f>IF(2&gt;Setup!$C$5,0,$G18*2/4*J18)</f>
         <v/>
       </c>
       <c r="O18" s="63">
-        <f>$H18*3/4*K18</f>
+        <f>IF(3&gt;Setup!$C$5,0,$G18*3/4*K18)</f>
         <v/>
       </c>
       <c r="P18" s="63">
-        <f>$H18*4/4*L18</f>
+        <f>IF(4&gt;Setup!$C$5,0,$G18*4/4*L18)</f>
         <v/>
       </c>
       <c r="Q18" s="83">
@@ -49703,7 +49703,7 @@
         <v/>
       </c>
       <c r="X18" s="84">
-        <f>$I18*W18</f>
+        <f>IF(Setup!$C$5&lt;4,0,$H18*W18)</f>
         <v/>
       </c>
       <c r="Y18" s="85">
@@ -49765,19 +49765,19 @@
         <v/>
       </c>
       <c r="M19" s="63">
-        <f>$H19*1/4*I19</f>
+        <f>IF(1&gt;Setup!$C$5,0,$G19*1/4*I19)</f>
         <v/>
       </c>
       <c r="N19" s="63">
-        <f>$H19*2/4*J19</f>
+        <f>IF(2&gt;Setup!$C$5,0,$G19*2/4*J19)</f>
         <v/>
       </c>
       <c r="O19" s="63">
-        <f>$H19*3/4*K19</f>
+        <f>IF(3&gt;Setup!$C$5,0,$G19*3/4*K19)</f>
         <v/>
       </c>
       <c r="P19" s="63">
-        <f>$H19*4/4*L19</f>
+        <f>IF(4&gt;Setup!$C$5,0,$G19*4/4*L19)</f>
         <v/>
       </c>
       <c r="Q19" s="83">
@@ -49809,7 +49809,7 @@
         <v/>
       </c>
       <c r="X19" s="84">
-        <f>$I19*W19</f>
+        <f>IF(Setup!$C$5&lt;4,0,$H19*W19)</f>
         <v/>
       </c>
       <c r="Y19" s="85">
@@ -49871,19 +49871,19 @@
         <v/>
       </c>
       <c r="M20" s="63">
-        <f>$H20*1/4*I20</f>
+        <f>IF(1&gt;Setup!$C$5,0,$G20*1/4*I20)</f>
         <v/>
       </c>
       <c r="N20" s="63">
-        <f>$H20*2/4*J20</f>
+        <f>IF(2&gt;Setup!$C$5,0,$G20*2/4*J20)</f>
         <v/>
       </c>
       <c r="O20" s="63">
-        <f>$H20*3/4*K20</f>
+        <f>IF(3&gt;Setup!$C$5,0,$G20*3/4*K20)</f>
         <v/>
       </c>
       <c r="P20" s="63">
-        <f>$H20*4/4*L20</f>
+        <f>IF(4&gt;Setup!$C$5,0,$G20*4/4*L20)</f>
         <v/>
       </c>
       <c r="Q20" s="83">
@@ -49915,7 +49915,7 @@
         <v/>
       </c>
       <c r="X20" s="84">
-        <f>$I20*W20</f>
+        <f>IF(Setup!$C$5&lt;4,0,$H20*W20)</f>
         <v/>
       </c>
       <c r="Y20" s="85">

</xml_diff>